<commit_message>
some changes in values in normal ranges
</commit_message>
<xml_diff>
--- a/Data Analysis & AI/tests/Data/normal ranges.xlsx
+++ b/Data Analysis & AI/tests/Data/normal ranges.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lenovo\EMAN\1.1.1 Graduation\Graduation-Project\Data Analysis &amp; AI\tests\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00AFFD4-A572-4342-B741-29872A875B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE73E69-F43E-4F8D-8AAF-4D2FF743A80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="6" xr2:uid="{BD5E39A0-6F15-4585-B47B-C3FEFEB75A9E}"/>
   </bookViews>
@@ -746,7 +746,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -774,6 +774,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -814,7 +820,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -829,12 +835,20 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1373,16 +1387,16 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="16" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1443,16 +1457,16 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="16" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1476,16 +1490,16 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="15" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1504,44 +1518,44 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="15" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="15" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="15" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1892,13 +1906,13 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="17" t="s">
         <v>102</v>
       </c>
       <c r="D5" s="10"/>
@@ -2016,35 +2030,37 @@
       <c r="E14" s="10"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="17" t="s">
         <v>110</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="17" t="s">
         <v>118</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="14" t="s">
         <v>119</v>
       </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
     </row>
@@ -2062,65 +2078,65 @@
       <c r="E18" s="10"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="17" t="s">
         <v>124</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="17" t="s">
         <v>126</v>
       </c>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="17" t="s">
         <v>128</v>
       </c>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="17" t="s">
         <v>130</v>
       </c>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="17" t="s">
         <v>132</v>
       </c>
       <c r="D23" s="10"/>

</xml_diff>